<commit_message>
Auto update Excel data tu Admin
</commit_message>
<xml_diff>
--- a/filetiendo.xlsx
+++ b/filetiendo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\viettel 2026\thang 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A046EBC-6D3F-4051-909A-A6209A3F9D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E19459-72BE-4896-8094-D18A401BB59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="808" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4556,41 +4556,17 @@
     <xf numFmtId="0" fontId="66" fillId="0" borderId="109" xfId="11" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="62" fillId="0" borderId="109" xfId="11" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="177" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="135" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="134" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="133" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="50" fillId="5" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="130" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="128" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="140" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="139" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="138" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="5" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="24" borderId="132" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4604,10 +4580,34 @@
     <xf numFmtId="0" fontId="17" fillId="5" borderId="129" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="135" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="134" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="133" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="16" borderId="136" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="2" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="140" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="139" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="138" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="67" fillId="18" borderId="165" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4679,16 +4679,16 @@
     <xf numFmtId="0" fontId="63" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="47" fillId="5" borderId="152" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="5" borderId="151" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="148" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="147" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="5" borderId="152" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="5" borderId="151" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="5" borderId="150" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4708,6 +4708,12 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="155" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="158" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="157" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="159" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4733,10 +4739,10 @@
     <xf numFmtId="0" fontId="55" fillId="0" borderId="164" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="158" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="69" fillId="29" borderId="165" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="157" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="69" fillId="29" borderId="165" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4761,12 +4767,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="168" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="69" fillId="29" borderId="165" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="29" borderId="165" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Comma" xfId="8" builtinId="3"/>
@@ -5656,166 +5656,166 @@
       </c>
     </row>
     <row r="2" spans="1:675" ht="23.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="210" t="s">
+      <c r="A2" s="200" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="86"/>
       <c r="C2" s="15"/>
-      <c r="D2" s="216" t="s">
+      <c r="D2" s="211" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="216"/>
-      <c r="F2" s="216"/>
-      <c r="G2" s="216"/>
-      <c r="H2" s="216"/>
-      <c r="I2" s="216"/>
-      <c r="J2" s="216"/>
-      <c r="K2" s="216"/>
-      <c r="L2" s="216"/>
-      <c r="M2" s="216"/>
-      <c r="N2" s="216"/>
-      <c r="O2" s="216"/>
-      <c r="P2" s="216"/>
-      <c r="Q2" s="216"/>
-      <c r="R2" s="216"/>
-      <c r="S2" s="216"/>
-      <c r="T2" s="214" t="s">
+      <c r="E2" s="211"/>
+      <c r="F2" s="211"/>
+      <c r="G2" s="211"/>
+      <c r="H2" s="211"/>
+      <c r="I2" s="211"/>
+      <c r="J2" s="211"/>
+      <c r="K2" s="211"/>
+      <c r="L2" s="211"/>
+      <c r="M2" s="211"/>
+      <c r="N2" s="211"/>
+      <c r="O2" s="211"/>
+      <c r="P2" s="211"/>
+      <c r="Q2" s="211"/>
+      <c r="R2" s="211"/>
+      <c r="S2" s="211"/>
+      <c r="T2" s="206" t="s">
         <v>36</v>
       </c>
-      <c r="U2" s="214"/>
-      <c r="V2" s="214"/>
-      <c r="W2" s="214"/>
-      <c r="X2" s="214"/>
-      <c r="Y2" s="214"/>
-      <c r="Z2" s="214"/>
-      <c r="AA2" s="214"/>
-      <c r="AB2" s="214"/>
-      <c r="AC2" s="214"/>
-      <c r="AD2" s="214"/>
-      <c r="AE2" s="214"/>
-      <c r="AF2" s="214"/>
-      <c r="AG2" s="214"/>
-      <c r="AH2" s="214"/>
-      <c r="AI2" s="214"/>
-      <c r="AJ2" s="213" t="s">
+      <c r="U2" s="206"/>
+      <c r="V2" s="206"/>
+      <c r="W2" s="206"/>
+      <c r="X2" s="206"/>
+      <c r="Y2" s="206"/>
+      <c r="Z2" s="206"/>
+      <c r="AA2" s="206"/>
+      <c r="AB2" s="206"/>
+      <c r="AC2" s="206"/>
+      <c r="AD2" s="206"/>
+      <c r="AE2" s="206"/>
+      <c r="AF2" s="206"/>
+      <c r="AG2" s="206"/>
+      <c r="AH2" s="206"/>
+      <c r="AI2" s="206"/>
+      <c r="AJ2" s="205" t="s">
         <v>37</v>
       </c>
-      <c r="AK2" s="213"/>
-      <c r="AL2" s="213"/>
-      <c r="AM2" s="213"/>
-      <c r="AN2" s="213"/>
-      <c r="AO2" s="213"/>
-      <c r="AP2" s="213"/>
-      <c r="AQ2" s="213"/>
-      <c r="AR2" s="213"/>
-      <c r="AS2" s="213"/>
-      <c r="AT2" s="213"/>
-      <c r="AU2" s="213"/>
-      <c r="AV2" s="212" t="s">
+      <c r="AK2" s="205"/>
+      <c r="AL2" s="205"/>
+      <c r="AM2" s="205"/>
+      <c r="AN2" s="205"/>
+      <c r="AO2" s="205"/>
+      <c r="AP2" s="205"/>
+      <c r="AQ2" s="205"/>
+      <c r="AR2" s="205"/>
+      <c r="AS2" s="205"/>
+      <c r="AT2" s="205"/>
+      <c r="AU2" s="205"/>
+      <c r="AV2" s="204" t="s">
         <v>38</v>
       </c>
-      <c r="AW2" s="212"/>
-      <c r="AX2" s="212"/>
-      <c r="AY2" s="212"/>
-      <c r="AZ2" s="212"/>
-      <c r="BA2" s="212"/>
-      <c r="BB2" s="212"/>
-      <c r="BC2" s="212"/>
-      <c r="BD2" s="212"/>
-      <c r="BE2" s="212"/>
-      <c r="BF2" s="212"/>
-      <c r="BG2" s="212"/>
+      <c r="AW2" s="204"/>
+      <c r="AX2" s="204"/>
+      <c r="AY2" s="204"/>
+      <c r="AZ2" s="204"/>
+      <c r="BA2" s="204"/>
+      <c r="BB2" s="204"/>
+      <c r="BC2" s="204"/>
+      <c r="BD2" s="204"/>
+      <c r="BE2" s="204"/>
+      <c r="BF2" s="204"/>
+      <c r="BG2" s="204"/>
     </row>
     <row r="3" spans="1:675" s="3" customFormat="1" ht="28.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="210"/>
-      <c r="B3" s="217" t="s">
+      <c r="A3" s="200"/>
+      <c r="B3" s="212" t="s">
         <v>39</v>
       </c>
       <c r="C3" s="87"/>
-      <c r="D3" s="204" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="205"/>
-      <c r="F3" s="205"/>
-      <c r="G3" s="205"/>
-      <c r="H3" s="204" t="s">
+      <c r="D3" s="202" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="203"/>
+      <c r="F3" s="203"/>
+      <c r="G3" s="203"/>
+      <c r="H3" s="202" t="s">
         <v>40</v>
       </c>
-      <c r="I3" s="205"/>
-      <c r="J3" s="205"/>
-      <c r="K3" s="205"/>
-      <c r="L3" s="204" t="s">
+      <c r="I3" s="203"/>
+      <c r="J3" s="203"/>
+      <c r="K3" s="203"/>
+      <c r="L3" s="202" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="205"/>
-      <c r="N3" s="205"/>
-      <c r="O3" s="205"/>
-      <c r="P3" s="207" t="s">
+      <c r="M3" s="203"/>
+      <c r="N3" s="203"/>
+      <c r="O3" s="203"/>
+      <c r="P3" s="215" t="s">
         <v>42</v>
       </c>
-      <c r="Q3" s="208"/>
-      <c r="R3" s="208"/>
-      <c r="S3" s="209"/>
-      <c r="T3" s="204" t="s">
+      <c r="Q3" s="216"/>
+      <c r="R3" s="216"/>
+      <c r="S3" s="217"/>
+      <c r="T3" s="202" t="s">
         <v>43</v>
       </c>
-      <c r="U3" s="205"/>
-      <c r="V3" s="205"/>
-      <c r="W3" s="205"/>
-      <c r="X3" s="204" t="s">
+      <c r="U3" s="203"/>
+      <c r="V3" s="203"/>
+      <c r="W3" s="203"/>
+      <c r="X3" s="202" t="s">
         <v>45</v>
       </c>
-      <c r="Y3" s="205"/>
-      <c r="Z3" s="205"/>
-      <c r="AA3" s="205"/>
-      <c r="AB3" s="204" t="s">
+      <c r="Y3" s="203"/>
+      <c r="Z3" s="203"/>
+      <c r="AA3" s="203"/>
+      <c r="AB3" s="202" t="s">
         <v>47</v>
       </c>
-      <c r="AC3" s="205"/>
-      <c r="AD3" s="205"/>
-      <c r="AE3" s="205"/>
-      <c r="AF3" s="204" t="s">
+      <c r="AC3" s="203"/>
+      <c r="AD3" s="203"/>
+      <c r="AE3" s="203"/>
+      <c r="AF3" s="202" t="s">
         <v>48</v>
       </c>
-      <c r="AG3" s="205"/>
-      <c r="AH3" s="205"/>
-      <c r="AI3" s="205"/>
-      <c r="AJ3" s="201" t="s">
+      <c r="AG3" s="203"/>
+      <c r="AH3" s="203"/>
+      <c r="AI3" s="203"/>
+      <c r="AJ3" s="208" t="s">
         <v>51</v>
       </c>
-      <c r="AK3" s="202"/>
-      <c r="AL3" s="202"/>
-      <c r="AM3" s="203"/>
-      <c r="AN3" s="201" t="s">
+      <c r="AK3" s="209"/>
+      <c r="AL3" s="209"/>
+      <c r="AM3" s="210"/>
+      <c r="AN3" s="208" t="s">
         <v>14</v>
       </c>
-      <c r="AO3" s="202"/>
-      <c r="AP3" s="202"/>
-      <c r="AQ3" s="203"/>
-      <c r="AR3" s="201" t="s">
+      <c r="AO3" s="209"/>
+      <c r="AP3" s="209"/>
+      <c r="AQ3" s="210"/>
+      <c r="AR3" s="208" t="s">
         <v>52</v>
       </c>
-      <c r="AS3" s="202"/>
-      <c r="AT3" s="202"/>
-      <c r="AU3" s="203"/>
-      <c r="AV3" s="205" t="s">
+      <c r="AS3" s="209"/>
+      <c r="AT3" s="209"/>
+      <c r="AU3" s="210"/>
+      <c r="AV3" s="203" t="s">
         <v>16</v>
       </c>
-      <c r="AW3" s="205"/>
-      <c r="AX3" s="205"/>
-      <c r="AY3" s="205"/>
-      <c r="AZ3" s="205" t="s">
+      <c r="AW3" s="203"/>
+      <c r="AX3" s="203"/>
+      <c r="AY3" s="203"/>
+      <c r="AZ3" s="203" t="s">
         <v>54</v>
       </c>
-      <c r="BA3" s="205"/>
-      <c r="BB3" s="205"/>
-      <c r="BC3" s="205"/>
-      <c r="BD3" s="204" t="s">
+      <c r="BA3" s="203"/>
+      <c r="BB3" s="203"/>
+      <c r="BC3" s="203"/>
+      <c r="BD3" s="202" t="s">
         <v>55</v>
       </c>
-      <c r="BE3" s="205"/>
-      <c r="BF3" s="215"/>
-      <c r="BG3" s="205"/>
+      <c r="BE3" s="203"/>
+      <c r="BF3" s="207"/>
+      <c r="BG3" s="203"/>
       <c r="BH3" s="2"/>
       <c r="BI3" s="2"/>
       <c r="BJ3" s="2"/>
@@ -6434,8 +6434,8 @@
       <c r="YY3" s="2"/>
     </row>
     <row r="4" spans="1:675" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="211"/>
-      <c r="B4" s="217"/>
+      <c r="A4" s="201"/>
+      <c r="B4" s="212"/>
       <c r="C4" s="88"/>
       <c r="D4" s="8" t="s">
         <v>2</v>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="AS5" s="129">
         <f>(VLOOKUP(B5,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.77680000000000005</v>
+        <v>0.78980000000000006</v>
       </c>
       <c r="AT5" s="14">
         <f t="shared" ref="AT5:AT18" si="20">IF(AS5&lt;94.5%,0,IF(AS5&lt;95.54%,50%,IF(AS5&lt;AR5,80%,100%+(30%*(AS5-AR5)/3.39%))))</f>
@@ -6788,7 +6788,7 @@
       </c>
       <c r="AU5" s="54">
         <f t="shared" ref="AU5:AU18" si="21">AR5-AS5</f>
-        <v>0.19319999999999993</v>
+        <v>0.18019999999999992</v>
       </c>
       <c r="AV5" s="57">
         <f>VLOOKUP(C5,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -7013,7 +7013,7 @@
       </c>
       <c r="AS6" s="129">
         <f>(VLOOKUP(B6,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.65590000000000004</v>
+        <v>0.68900000000000006</v>
       </c>
       <c r="AT6" s="14">
         <f t="shared" si="20"/>
@@ -7021,7 +7021,7 @@
       </c>
       <c r="AU6" s="54">
         <f t="shared" si="21"/>
-        <v>0.31409999999999993</v>
+        <v>0.28099999999999992</v>
       </c>
       <c r="AV6" s="57">
         <f>VLOOKUP(C6,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AS7" s="129">
         <f>(VLOOKUP(B7,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.73170000000000002</v>
+        <v>0.75019999999999998</v>
       </c>
       <c r="AT7" s="14">
         <f t="shared" si="20"/>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="AU7" s="54">
         <f t="shared" si="21"/>
-        <v>0.23829999999999996</v>
+        <v>0.2198</v>
       </c>
       <c r="AV7" s="57">
         <f>VLOOKUP(C7,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="AS8" s="129">
         <f>(VLOOKUP(B8,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.30780000000000002</v>
+        <v>0.31659999999999999</v>
       </c>
       <c r="AT8" s="14">
         <f t="shared" si="20"/>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="AU8" s="54">
         <f t="shared" si="21"/>
-        <v>0.6621999999999999</v>
+        <v>0.65339999999999998</v>
       </c>
       <c r="AV8" s="57">
         <f>VLOOKUP(C8,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -7712,7 +7712,7 @@
       </c>
       <c r="AS9" s="129">
         <f>(VLOOKUP(B9,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.54569999999999996</v>
+        <v>0.56869999999999998</v>
       </c>
       <c r="AT9" s="14">
         <f t="shared" si="20"/>
@@ -7720,7 +7720,7 @@
       </c>
       <c r="AU9" s="54">
         <f t="shared" si="21"/>
-        <v>0.42430000000000001</v>
+        <v>0.40129999999999999</v>
       </c>
       <c r="AV9" s="57">
         <f>VLOOKUP(C9,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -7945,7 +7945,7 @@
       </c>
       <c r="AS10" s="129">
         <f>(VLOOKUP(B10,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.51470000000000005</v>
+        <v>0.55700000000000005</v>
       </c>
       <c r="AT10" s="14">
         <f t="shared" si="20"/>
@@ -7953,7 +7953,7 @@
       </c>
       <c r="AU10" s="54">
         <f t="shared" si="21"/>
-        <v>0.45529999999999993</v>
+        <v>0.41299999999999992</v>
       </c>
       <c r="AV10" s="57">
         <f>VLOOKUP(C10,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -8178,7 +8178,7 @@
       </c>
       <c r="AS11" s="129">
         <f>(VLOOKUP(B11,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.623</v>
+        <v>0.6412000000000001</v>
       </c>
       <c r="AT11" s="14">
         <f t="shared" si="20"/>
@@ -8186,7 +8186,7 @@
       </c>
       <c r="AU11" s="54">
         <f t="shared" si="21"/>
-        <v>0.34699999999999998</v>
+        <v>0.32879999999999987</v>
       </c>
       <c r="AV11" s="57">
         <f>VLOOKUP(C11,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="AS12" s="129">
         <f>(VLOOKUP(B12,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.58150000000000002</v>
+        <v>0.58609999999999995</v>
       </c>
       <c r="AT12" s="14">
         <f t="shared" si="20"/>
@@ -8419,7 +8419,7 @@
       </c>
       <c r="AU12" s="54">
         <f t="shared" si="21"/>
-        <v>0.38849999999999996</v>
+        <v>0.38390000000000002</v>
       </c>
       <c r="AV12" s="57">
         <f>VLOOKUP(C12,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -8644,7 +8644,7 @@
       </c>
       <c r="AS13" s="129">
         <f>(VLOOKUP(B13,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.74010000000000009</v>
+        <v>0.77280000000000004</v>
       </c>
       <c r="AT13" s="14">
         <f t="shared" si="20"/>
@@ -8652,7 +8652,7 @@
       </c>
       <c r="AU13" s="54">
         <f t="shared" si="21"/>
-        <v>0.22989999999999988</v>
+        <v>0.19719999999999993</v>
       </c>
       <c r="AV13" s="57">
         <f>VLOOKUP(C13,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -8877,7 +8877,7 @@
       </c>
       <c r="AS14" s="129">
         <f>(VLOOKUP(B14,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.56110000000000004</v>
+        <v>0.5756</v>
       </c>
       <c r="AT14" s="14">
         <f t="shared" si="20"/>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="AU14" s="54">
         <f t="shared" si="21"/>
-        <v>0.40889999999999993</v>
+        <v>0.39439999999999997</v>
       </c>
       <c r="AV14" s="57">
         <f>VLOOKUP(C14,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -9110,7 +9110,7 @@
       </c>
       <c r="AS15" s="129">
         <f>(VLOOKUP(B15,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.62829999999999997</v>
+        <v>0.64300000000000002</v>
       </c>
       <c r="AT15" s="14">
         <f t="shared" si="20"/>
@@ -9118,7 +9118,7 @@
       </c>
       <c r="AU15" s="54">
         <f t="shared" si="21"/>
-        <v>0.3417</v>
+        <v>0.32699999999999996</v>
       </c>
       <c r="AV15" s="57">
         <f>VLOOKUP(C15,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="AS16" s="129">
         <f>(VLOOKUP(B16,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.69769999999999999</v>
+        <v>0.71420000000000006</v>
       </c>
       <c r="AT16" s="14">
         <f t="shared" si="20"/>
@@ -9351,7 +9351,7 @@
       </c>
       <c r="AU16" s="54">
         <f t="shared" si="21"/>
-        <v>0.27229999999999999</v>
+        <v>0.25579999999999992</v>
       </c>
       <c r="AV16" s="57">
         <f>VLOOKUP(C16,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -9576,7 +9576,7 @@
       </c>
       <c r="AS17" s="129">
         <f>(VLOOKUP(B17,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.7409</v>
+        <v>0.75930000000000009</v>
       </c>
       <c r="AT17" s="14">
         <f t="shared" si="20"/>
@@ -9584,7 +9584,7 @@
       </c>
       <c r="AU17" s="54">
         <f t="shared" si="21"/>
-        <v>0.22909999999999997</v>
+        <v>0.21069999999999989</v>
       </c>
       <c r="AV17" s="57">
         <f>VLOOKUP(C17,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -9809,7 +9809,7 @@
       </c>
       <c r="AS18" s="129">
         <f>(VLOOKUP(B18,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.72129999999999994</v>
+        <v>0.73239999999999994</v>
       </c>
       <c r="AT18" s="14">
         <f t="shared" si="20"/>
@@ -9817,7 +9817,7 @@
       </c>
       <c r="AU18" s="54">
         <f t="shared" si="21"/>
-        <v>0.24870000000000003</v>
+        <v>0.23760000000000003</v>
       </c>
       <c r="AV18" s="57">
         <f>VLOOKUP(C18,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -9874,11 +9874,11 @@
       <c r="C19" s="15"/>
       <c r="D19" s="15"/>
       <c r="E19" s="16"/>
-      <c r="F19" s="200">
+      <c r="F19" s="213">
         <f ca="1">TODAY()</f>
         <v>46076</v>
       </c>
-      <c r="G19" s="200"/>
+      <c r="G19" s="213"/>
       <c r="H19" s="90"/>
       <c r="I19" s="91">
         <f ca="1">DAY(F19)</f>
@@ -9891,33 +9891,33 @@
         <f ca="1">I19/J19</f>
         <v>0.74193548387096775</v>
       </c>
-      <c r="L19" s="206" t="s">
+      <c r="L19" s="214" t="s">
         <v>124</v>
       </c>
-      <c r="M19" s="206"/>
-      <c r="N19" s="206"/>
-      <c r="O19" s="206"/>
-      <c r="P19" s="206"/>
-      <c r="Q19" s="206"/>
-      <c r="R19" s="206"/>
-      <c r="S19" s="206"/>
-      <c r="T19" s="206"/>
-      <c r="U19" s="206"/>
-      <c r="V19" s="206"/>
-      <c r="W19" s="206"/>
-      <c r="X19" s="206"/>
-      <c r="Y19" s="206"/>
-      <c r="Z19" s="206"/>
-      <c r="AA19" s="206"/>
-      <c r="AB19" s="206"/>
-      <c r="AC19" s="206"/>
-      <c r="AD19" s="206"/>
-      <c r="AE19" s="206"/>
-      <c r="AF19" s="206"/>
-      <c r="AG19" s="206"/>
-      <c r="AH19" s="206"/>
-      <c r="AI19" s="206"/>
-      <c r="AJ19" s="206"/>
+      <c r="M19" s="214"/>
+      <c r="N19" s="214"/>
+      <c r="O19" s="214"/>
+      <c r="P19" s="214"/>
+      <c r="Q19" s="214"/>
+      <c r="R19" s="214"/>
+      <c r="S19" s="214"/>
+      <c r="T19" s="214"/>
+      <c r="U19" s="214"/>
+      <c r="V19" s="214"/>
+      <c r="W19" s="214"/>
+      <c r="X19" s="214"/>
+      <c r="Y19" s="214"/>
+      <c r="Z19" s="214"/>
+      <c r="AA19" s="214"/>
+      <c r="AB19" s="214"/>
+      <c r="AC19" s="214"/>
+      <c r="AD19" s="214"/>
+      <c r="AE19" s="214"/>
+      <c r="AF19" s="214"/>
+      <c r="AG19" s="214"/>
+      <c r="AH19" s="214"/>
+      <c r="AI19" s="214"/>
+      <c r="AJ19" s="214"/>
       <c r="AK19" s="16"/>
       <c r="AL19" s="32"/>
       <c r="AM19" s="16"/>
@@ -10110,6 +10110,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="AN3:AQ3"/>
+    <mergeCell ref="AF3:AI3"/>
+    <mergeCell ref="L19:AJ19"/>
+    <mergeCell ref="P3:S3"/>
+    <mergeCell ref="T3:W3"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="X3:AA3"/>
     <mergeCell ref="AV2:BG2"/>
@@ -10126,12 +10132,6 @@
     <mergeCell ref="D3:G3"/>
     <mergeCell ref="H3:K3"/>
     <mergeCell ref="L3:O3"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="AN3:AQ3"/>
-    <mergeCell ref="AF3:AI3"/>
-    <mergeCell ref="L19:AJ19"/>
-    <mergeCell ref="P3:S3"/>
-    <mergeCell ref="T3:W3"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="C3:C4">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="D14" s="74">
         <f>VLOOKUP($B$2,'TH NV'!$A$5:$BG$18,N14,0)</f>
-        <v>0.77680000000000005</v>
+        <v>0.78980000000000006</v>
       </c>
       <c r="E14" s="49" t="e">
         <f>VLOOKUP($B$2,'TH NV'!$A$1:$BG$18,70,0)</f>
@@ -11170,7 +11170,7 @@
       </c>
       <c r="J14" s="65">
         <f t="shared" si="2"/>
-        <v>0.19319999999999993</v>
+        <v>0.18019999999999992</v>
       </c>
       <c r="K14" s="222"/>
       <c r="L14" s="114" t="s">
@@ -11351,42 +11351,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" s="1" customFormat="1" ht="24.75" x14ac:dyDescent="0.45">
-      <c r="D1" s="216" t="s">
+      <c r="D1" s="211" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="216"/>
-      <c r="F1" s="216"/>
-      <c r="G1" s="216"/>
-      <c r="H1" s="216"/>
-      <c r="I1" s="216"/>
-      <c r="J1" s="216"/>
-      <c r="K1" s="216"/>
-      <c r="L1" s="216"/>
-      <c r="M1" s="216"/>
-      <c r="N1" s="216"/>
-      <c r="O1" s="216"/>
-      <c r="P1" s="216"/>
-      <c r="Q1" s="216"/>
-      <c r="R1" s="216"/>
-      <c r="S1" s="216"/>
-      <c r="T1" s="214" t="s">
+      <c r="E1" s="211"/>
+      <c r="F1" s="211"/>
+      <c r="G1" s="211"/>
+      <c r="H1" s="211"/>
+      <c r="I1" s="211"/>
+      <c r="J1" s="211"/>
+      <c r="K1" s="211"/>
+      <c r="L1" s="211"/>
+      <c r="M1" s="211"/>
+      <c r="N1" s="211"/>
+      <c r="O1" s="211"/>
+      <c r="P1" s="211"/>
+      <c r="Q1" s="211"/>
+      <c r="R1" s="211"/>
+      <c r="S1" s="211"/>
+      <c r="T1" s="206" t="s">
         <v>36</v>
       </c>
-      <c r="U1" s="214"/>
-      <c r="V1" s="214"/>
-      <c r="W1" s="214"/>
-      <c r="X1" s="214"/>
-      <c r="Y1" s="214"/>
-      <c r="Z1" s="214"/>
-      <c r="AA1" s="214"/>
-      <c r="AB1" s="214"/>
-      <c r="AC1" s="214"/>
-      <c r="AD1" s="214"/>
-      <c r="AE1" s="214"/>
-      <c r="AF1" s="214"/>
-      <c r="AG1" s="214"/>
-      <c r="AH1" s="214"/>
-      <c r="AI1" s="214"/>
+      <c r="U1" s="206"/>
+      <c r="V1" s="206"/>
+      <c r="W1" s="206"/>
+      <c r="X1" s="206"/>
+      <c r="Y1" s="206"/>
+      <c r="Z1" s="206"/>
+      <c r="AA1" s="206"/>
+      <c r="AB1" s="206"/>
+      <c r="AC1" s="206"/>
+      <c r="AD1" s="206"/>
+      <c r="AE1" s="206"/>
+      <c r="AF1" s="206"/>
+      <c r="AG1" s="206"/>
+      <c r="AH1" s="206"/>
+      <c r="AI1" s="206"/>
       <c r="AJ1" s="234" t="s">
         <v>37</v>
       </c>
@@ -11419,90 +11419,90 @@
     <row r="2" spans="1:59" ht="15.6" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="204" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="205"/>
-      <c r="F2" s="205"/>
-      <c r="G2" s="205"/>
-      <c r="H2" s="204" t="s">
+      <c r="D2" s="202" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="203"/>
+      <c r="F2" s="203"/>
+      <c r="G2" s="203"/>
+      <c r="H2" s="202" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="205"/>
-      <c r="J2" s="205"/>
-      <c r="K2" s="205"/>
-      <c r="L2" s="204" t="s">
+      <c r="I2" s="203"/>
+      <c r="J2" s="203"/>
+      <c r="K2" s="203"/>
+      <c r="L2" s="202" t="s">
         <v>41</v>
       </c>
-      <c r="M2" s="205"/>
-      <c r="N2" s="205"/>
-      <c r="O2" s="205"/>
-      <c r="P2" s="207" t="s">
+      <c r="M2" s="203"/>
+      <c r="N2" s="203"/>
+      <c r="O2" s="203"/>
+      <c r="P2" s="215" t="s">
         <v>42</v>
       </c>
-      <c r="Q2" s="208"/>
-      <c r="R2" s="208"/>
-      <c r="S2" s="209"/>
-      <c r="T2" s="204" t="s">
+      <c r="Q2" s="216"/>
+      <c r="R2" s="216"/>
+      <c r="S2" s="217"/>
+      <c r="T2" s="202" t="s">
         <v>43</v>
       </c>
-      <c r="U2" s="205"/>
-      <c r="V2" s="205"/>
-      <c r="W2" s="205"/>
-      <c r="X2" s="204" t="s">
+      <c r="U2" s="203"/>
+      <c r="V2" s="203"/>
+      <c r="W2" s="203"/>
+      <c r="X2" s="202" t="s">
         <v>45</v>
       </c>
-      <c r="Y2" s="205"/>
-      <c r="Z2" s="205"/>
-      <c r="AA2" s="205"/>
-      <c r="AB2" s="204" t="s">
+      <c r="Y2" s="203"/>
+      <c r="Z2" s="203"/>
+      <c r="AA2" s="203"/>
+      <c r="AB2" s="202" t="s">
         <v>47</v>
       </c>
-      <c r="AC2" s="205"/>
-      <c r="AD2" s="205"/>
-      <c r="AE2" s="205"/>
-      <c r="AF2" s="204" t="s">
+      <c r="AC2" s="203"/>
+      <c r="AD2" s="203"/>
+      <c r="AE2" s="203"/>
+      <c r="AF2" s="202" t="s">
         <v>48</v>
       </c>
-      <c r="AG2" s="205"/>
-      <c r="AH2" s="205"/>
-      <c r="AI2" s="205"/>
-      <c r="AJ2" s="201" t="s">
+      <c r="AG2" s="203"/>
+      <c r="AH2" s="203"/>
+      <c r="AI2" s="203"/>
+      <c r="AJ2" s="208" t="s">
         <v>51</v>
       </c>
-      <c r="AK2" s="202"/>
-      <c r="AL2" s="202"/>
-      <c r="AM2" s="203"/>
-      <c r="AN2" s="201" t="s">
+      <c r="AK2" s="209"/>
+      <c r="AL2" s="209"/>
+      <c r="AM2" s="210"/>
+      <c r="AN2" s="208" t="s">
         <v>14</v>
       </c>
-      <c r="AO2" s="202"/>
-      <c r="AP2" s="202"/>
-      <c r="AQ2" s="203"/>
-      <c r="AR2" s="201" t="s">
+      <c r="AO2" s="209"/>
+      <c r="AP2" s="209"/>
+      <c r="AQ2" s="210"/>
+      <c r="AR2" s="208" t="s">
         <v>52</v>
       </c>
-      <c r="AS2" s="202"/>
-      <c r="AT2" s="202"/>
-      <c r="AU2" s="203"/>
-      <c r="AV2" s="205" t="s">
+      <c r="AS2" s="209"/>
+      <c r="AT2" s="209"/>
+      <c r="AU2" s="210"/>
+      <c r="AV2" s="203" t="s">
         <v>16</v>
       </c>
-      <c r="AW2" s="205"/>
-      <c r="AX2" s="205"/>
-      <c r="AY2" s="205"/>
-      <c r="AZ2" s="205" t="s">
+      <c r="AW2" s="203"/>
+      <c r="AX2" s="203"/>
+      <c r="AY2" s="203"/>
+      <c r="AZ2" s="203" t="s">
         <v>54</v>
       </c>
-      <c r="BA2" s="205"/>
-      <c r="BB2" s="205"/>
-      <c r="BC2" s="205"/>
-      <c r="BD2" s="204" t="s">
+      <c r="BA2" s="203"/>
+      <c r="BB2" s="203"/>
+      <c r="BC2" s="203"/>
+      <c r="BD2" s="202" t="s">
         <v>55</v>
       </c>
-      <c r="BE2" s="205"/>
-      <c r="BF2" s="215"/>
-      <c r="BG2" s="205"/>
+      <c r="BE2" s="203"/>
+      <c r="BF2" s="207"/>
+      <c r="BG2" s="203"/>
     </row>
     <row r="3" spans="1:59" ht="15" x14ac:dyDescent="0.45">
       <c r="B3" s="8" t="s">
@@ -11855,7 +11855,7 @@
       </c>
       <c r="AS4" s="129">
         <f>(VLOOKUP(B4,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.77680000000000005</v>
+        <v>0.78980000000000006</v>
       </c>
       <c r="AT4" s="14">
         <f t="shared" ref="AT4" si="20">IF(AS4&lt;94.5%,0,IF(AS4&lt;95.54%,50%,IF(AS4&lt;AR4,80%,100%+(30%*(AS4-AR4)/3.39%))))</f>
@@ -11863,7 +11863,7 @@
       </c>
       <c r="AU4" s="54">
         <f t="shared" ref="AU4" si="21">AR4-AS4</f>
-        <v>0.19319999999999993</v>
+        <v>0.18019999999999992</v>
       </c>
       <c r="AV4" s="57">
         <f>VLOOKUP(A4,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -12089,7 +12089,7 @@
       </c>
       <c r="AS5" s="129">
         <f>(VLOOKUP(B5,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.623</v>
+        <v>0.6412000000000001</v>
       </c>
       <c r="AT5" s="14">
         <f t="shared" ref="AT5:AT16" si="48">IF(AS5&lt;94.5%,0,IF(AS5&lt;95.54%,50%,IF(AS5&lt;AR5,80%,100%+(30%*(AS5-AR5)/3.39%))))</f>
@@ -12097,7 +12097,7 @@
       </c>
       <c r="AU5" s="54">
         <f t="shared" ref="AU5:AU16" si="49">AR5-AS5</f>
-        <v>0.34699999999999998</v>
+        <v>0.32879999999999987</v>
       </c>
       <c r="AV5" s="57">
         <f>VLOOKUP(A5,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -12323,7 +12323,7 @@
       </c>
       <c r="AS6" s="129">
         <f>(VLOOKUP(B6,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.58150000000000002</v>
+        <v>0.58609999999999995</v>
       </c>
       <c r="AT6" s="14">
         <f t="shared" si="48"/>
@@ -12331,7 +12331,7 @@
       </c>
       <c r="AU6" s="54">
         <f t="shared" si="49"/>
-        <v>0.38849999999999996</v>
+        <v>0.38390000000000002</v>
       </c>
       <c r="AV6" s="57">
         <f>VLOOKUP(A6,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -12557,7 +12557,7 @@
       </c>
       <c r="AS7" s="129">
         <f>(VLOOKUP(B7,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.56110000000000004</v>
+        <v>0.5756</v>
       </c>
       <c r="AT7" s="14">
         <f t="shared" si="48"/>
@@ -12565,7 +12565,7 @@
       </c>
       <c r="AU7" s="54">
         <f t="shared" si="49"/>
-        <v>0.40889999999999993</v>
+        <v>0.39439999999999997</v>
       </c>
       <c r="AV7" s="57">
         <f>VLOOKUP(A7,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -12791,7 +12791,7 @@
       </c>
       <c r="AS8" s="129">
         <f>(VLOOKUP(B8,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.69769999999999999</v>
+        <v>0.71420000000000006</v>
       </c>
       <c r="AT8" s="14">
         <f t="shared" si="48"/>
@@ -12799,7 +12799,7 @@
       </c>
       <c r="AU8" s="54">
         <f t="shared" si="49"/>
-        <v>0.27229999999999999</v>
+        <v>0.25579999999999992</v>
       </c>
       <c r="AV8" s="57">
         <f>VLOOKUP(A8,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -13086,7 +13086,7 @@
       </c>
       <c r="AS10" s="129">
         <f>(VLOOKUP(B10,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.65590000000000004</v>
+        <v>0.68900000000000006</v>
       </c>
       <c r="AT10" s="14">
         <f t="shared" si="48"/>
@@ -13094,7 +13094,7 @@
       </c>
       <c r="AU10" s="54">
         <f t="shared" si="49"/>
-        <v>0.31409999999999993</v>
+        <v>0.28099999999999992</v>
       </c>
       <c r="AV10" s="57">
         <f>VLOOKUP(A10,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -13320,7 +13320,7 @@
       </c>
       <c r="AS11" s="129">
         <f>(VLOOKUP(B11,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.73170000000000002</v>
+        <v>0.75019999999999998</v>
       </c>
       <c r="AT11" s="14">
         <f t="shared" si="48"/>
@@ -13328,7 +13328,7 @@
       </c>
       <c r="AU11" s="54">
         <f t="shared" si="49"/>
-        <v>0.23829999999999996</v>
+        <v>0.2198</v>
       </c>
       <c r="AV11" s="57">
         <f>VLOOKUP(A11,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -13554,7 +13554,7 @@
       </c>
       <c r="AS12" s="129">
         <f>(VLOOKUP(B12,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.30780000000000002</v>
+        <v>0.31659999999999999</v>
       </c>
       <c r="AT12" s="14">
         <f t="shared" si="48"/>
@@ -13562,7 +13562,7 @@
       </c>
       <c r="AU12" s="54">
         <f t="shared" si="49"/>
-        <v>0.6621999999999999</v>
+        <v>0.65339999999999998</v>
       </c>
       <c r="AV12" s="57">
         <f>VLOOKUP(A12,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="AS13" s="129">
         <f>(VLOOKUP(B13,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.51470000000000005</v>
+        <v>0.55700000000000005</v>
       </c>
       <c r="AT13" s="14">
         <f t="shared" si="48"/>
@@ -13796,7 +13796,7 @@
       </c>
       <c r="AU13" s="54">
         <f t="shared" si="49"/>
-        <v>0.45529999999999993</v>
+        <v>0.41299999999999992</v>
       </c>
       <c r="AV13" s="57">
         <f>VLOOKUP(A13,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -14022,7 +14022,7 @@
       </c>
       <c r="AS14" s="129">
         <f>(VLOOKUP(B14,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.74010000000000009</v>
+        <v>0.77280000000000004</v>
       </c>
       <c r="AT14" s="14">
         <f t="shared" si="48"/>
@@ -14030,7 +14030,7 @@
       </c>
       <c r="AU14" s="54">
         <f t="shared" si="49"/>
-        <v>0.22989999999999988</v>
+        <v>0.19719999999999993</v>
       </c>
       <c r="AV14" s="57">
         <f>VLOOKUP(A14,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -14256,7 +14256,7 @@
       </c>
       <c r="AS15" s="129">
         <f>(VLOOKUP(B15,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.62829999999999997</v>
+        <v>0.64300000000000002</v>
       </c>
       <c r="AT15" s="14">
         <f t="shared" si="48"/>
@@ -14264,7 +14264,7 @@
       </c>
       <c r="AU15" s="54">
         <f t="shared" si="49"/>
-        <v>0.3417</v>
+        <v>0.32699999999999996</v>
       </c>
       <c r="AV15" s="57">
         <f>VLOOKUP(A15,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -14490,7 +14490,7 @@
       </c>
       <c r="AS16" s="129">
         <f>(VLOOKUP(B16,cuoc!$B$7:$P$27,14,0))*1%</f>
-        <v>0.7409</v>
+        <v>0.75930000000000009</v>
       </c>
       <c r="AT16" s="14">
         <f t="shared" si="48"/>
@@ -14498,7 +14498,7 @@
       </c>
       <c r="AU16" s="54">
         <f t="shared" si="49"/>
-        <v>0.22909999999999997</v>
+        <v>0.21069999999999989</v>
       </c>
       <c r="AV16" s="57">
         <f>VLOOKUP(A16,'Giao CT'!$D$6:$S$20,14,0)</f>
@@ -14582,11 +14582,11 @@
       </c>
       <c r="C19" s="142">
         <f ca="1">SUMIF(cuoc!A7:P27,'tiến độ'!A19,cuoc!M7:M27)</f>
-        <v>417352699</v>
+        <v>426159900</v>
       </c>
       <c r="D19" s="142">
         <f ca="1">B19*0.968-C19</f>
-        <v>205821372.25599992</v>
+        <v>197014171.25599992</v>
       </c>
       <c r="E19" s="137"/>
       <c r="H19" s="137"/>
@@ -14603,11 +14603,11 @@
       </c>
       <c r="C20" s="143">
         <f ca="1">SUMIF(cuoc!A8:P27,'tiến độ'!A20,cuoc!M8:M27)</f>
-        <v>663687252</v>
+        <v>688184642</v>
       </c>
       <c r="D20" s="142">
         <f ca="1">B20*0.968-C20</f>
-        <v>280296674.77600002</v>
+        <v>255799284.77600002</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.45">
@@ -14793,6 +14793,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="D1:S1"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="P2:S2"/>
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
     <mergeCell ref="AF2:AI2"/>
@@ -14806,11 +14811,6 @@
     <mergeCell ref="AJ2:AM2"/>
     <mergeCell ref="AN2:AQ2"/>
     <mergeCell ref="T2:W2"/>
-    <mergeCell ref="D1:S1"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="P2:S2"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="F4:F16">
@@ -23286,6 +23286,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="X5:AE5"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="H5:O5"/>
+    <mergeCell ref="P5:W5"/>
     <mergeCell ref="CB5:CI5"/>
     <mergeCell ref="CJ5:CQ5"/>
     <mergeCell ref="CR5:CY5"/>
@@ -23296,12 +23302,6 @@
     <mergeCell ref="BD5:BK5"/>
     <mergeCell ref="BL5:BS5"/>
     <mergeCell ref="BT5:CA5"/>
-    <mergeCell ref="X5:AE5"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="H5:O5"/>
-    <mergeCell ref="P5:W5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23399,7 +23399,7 @@
       <c r="A3" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="245" t="s">
+      <c r="B3" s="243" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="101" t="s">
@@ -23411,70 +23411,70 @@
       <c r="E3" s="247" t="s">
         <v>202</v>
       </c>
-      <c r="F3" s="243" t="s">
+      <c r="F3" s="245" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="243" t="s">
+      <c r="G3" s="245" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="243" t="s">
+      <c r="H3" s="245" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="243" t="s">
+      <c r="I3" s="245" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="243" t="s">
+      <c r="J3" s="245" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="243" t="s">
+      <c r="K3" s="245" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="243" t="s">
+      <c r="L3" s="245" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="243" t="s">
+      <c r="M3" s="245" t="s">
         <v>203</v>
       </c>
-      <c r="N3" s="243" t="s">
+      <c r="N3" s="245" t="s">
         <v>286</v>
       </c>
-      <c r="O3" s="243" t="s">
+      <c r="O3" s="245" t="s">
         <v>14</v>
       </c>
-      <c r="P3" s="243" t="s">
+      <c r="P3" s="245" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="243" t="s">
+      <c r="Q3" s="245" t="s">
         <v>16</v>
       </c>
-      <c r="R3" s="243" t="s">
+      <c r="R3" s="245" t="s">
         <v>17</v>
       </c>
-      <c r="S3" s="243" t="s">
+      <c r="S3" s="245" t="s">
         <v>18</v>
       </c>
       <c r="T3" s="99"/>
     </row>
     <row r="4" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="100"/>
-      <c r="B4" s="246"/>
+      <c r="B4" s="244"/>
       <c r="C4" s="101"/>
       <c r="D4" s="101"/>
       <c r="E4" s="248"/>
-      <c r="F4" s="244"/>
-      <c r="G4" s="244"/>
-      <c r="H4" s="244"/>
-      <c r="I4" s="244"/>
-      <c r="J4" s="244"/>
-      <c r="K4" s="244"/>
-      <c r="L4" s="244"/>
-      <c r="M4" s="244"/>
-      <c r="N4" s="244"/>
-      <c r="O4" s="244"/>
-      <c r="P4" s="244"/>
-      <c r="Q4" s="244"/>
-      <c r="R4" s="244"/>
-      <c r="S4" s="244"/>
+      <c r="F4" s="246"/>
+      <c r="G4" s="246"/>
+      <c r="H4" s="246"/>
+      <c r="I4" s="246"/>
+      <c r="J4" s="246"/>
+      <c r="K4" s="246"/>
+      <c r="L4" s="246"/>
+      <c r="M4" s="246"/>
+      <c r="N4" s="246"/>
+      <c r="O4" s="246"/>
+      <c r="P4" s="246"/>
+      <c r="Q4" s="246"/>
+      <c r="R4" s="246"/>
+      <c r="S4" s="246"/>
       <c r="T4" s="99"/>
     </row>
     <row r="5" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.45">
@@ -24792,6 +24792,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="R3:R4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="H3:H4"/>
@@ -24802,12 +24808,6 @@
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="S3:S4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="R3:R4"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.69991251615088756" right="0.69991251615088756" top="0.74990626395218019" bottom="0.74990626395218019" header="0.29996251027415122" footer="0.29996251027415122"/>
@@ -26083,68 +26083,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:48" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="256" t="s">
+      <c r="A1" s="258" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="256"/>
-      <c r="C1" s="256"/>
-      <c r="D1" s="256"/>
-      <c r="E1" s="256"/>
-      <c r="F1" s="256"/>
-      <c r="G1" s="256"/>
-      <c r="H1" s="256"/>
-      <c r="I1" s="256"/>
-      <c r="J1" s="256"/>
-      <c r="K1" s="256"/>
-      <c r="M1" s="259" t="s">
+      <c r="B1" s="258"/>
+      <c r="C1" s="258"/>
+      <c r="D1" s="258"/>
+      <c r="E1" s="258"/>
+      <c r="F1" s="258"/>
+      <c r="G1" s="258"/>
+      <c r="H1" s="258"/>
+      <c r="I1" s="258"/>
+      <c r="J1" s="258"/>
+      <c r="K1" s="258"/>
+      <c r="M1" s="261" t="s">
         <v>241</v>
       </c>
-      <c r="N1" s="259"/>
-      <c r="O1" s="259"/>
-      <c r="P1" s="259"/>
-      <c r="Q1" s="259"/>
-      <c r="R1" s="259"/>
-      <c r="S1" s="259"/>
-      <c r="T1" s="259"/>
-      <c r="U1" s="259"/>
-      <c r="V1" s="259"/>
-      <c r="W1" s="259"/>
-      <c r="X1" s="259"/>
-      <c r="Y1" s="259"/>
-      <c r="Z1" s="259"/>
+      <c r="N1" s="261"/>
+      <c r="O1" s="261"/>
+      <c r="P1" s="261"/>
+      <c r="Q1" s="261"/>
+      <c r="R1" s="261"/>
+      <c r="S1" s="261"/>
+      <c r="T1" s="261"/>
+      <c r="U1" s="261"/>
+      <c r="V1" s="261"/>
+      <c r="W1" s="261"/>
+      <c r="X1" s="261"/>
+      <c r="Y1" s="261"/>
+      <c r="Z1" s="261"/>
     </row>
     <row r="2" spans="1:48" ht="24.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="257"/>
-      <c r="B2" s="257"/>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="257"/>
-      <c r="H2" s="257"/>
-      <c r="I2" s="257"/>
-      <c r="J2" s="257"/>
-      <c r="K2" s="257"/>
-      <c r="M2" s="260"/>
-      <c r="N2" s="260"/>
-      <c r="O2" s="260"/>
-      <c r="P2" s="260"/>
-      <c r="Q2" s="260"/>
-      <c r="R2" s="260"/>
-      <c r="S2" s="260"/>
-      <c r="T2" s="260"/>
-      <c r="U2" s="260"/>
-      <c r="V2" s="260"/>
-      <c r="W2" s="260"/>
-      <c r="X2" s="260"/>
-      <c r="Y2" s="260"/>
-      <c r="Z2" s="260"/>
+      <c r="A2" s="259"/>
+      <c r="B2" s="259"/>
+      <c r="C2" s="259"/>
+      <c r="D2" s="259"/>
+      <c r="E2" s="259"/>
+      <c r="F2" s="259"/>
+      <c r="G2" s="259"/>
+      <c r="H2" s="259"/>
+      <c r="I2" s="259"/>
+      <c r="J2" s="259"/>
+      <c r="K2" s="259"/>
+      <c r="M2" s="262"/>
+      <c r="N2" s="262"/>
+      <c r="O2" s="262"/>
+      <c r="P2" s="262"/>
+      <c r="Q2" s="262"/>
+      <c r="R2" s="262"/>
+      <c r="S2" s="262"/>
+      <c r="T2" s="262"/>
+      <c r="U2" s="262"/>
+      <c r="V2" s="262"/>
+      <c r="W2" s="262"/>
+      <c r="X2" s="262"/>
+      <c r="Y2" s="262"/>
+      <c r="Z2" s="262"/>
     </row>
     <row r="3" spans="1:48" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="253" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="254" t="s">
+      <c r="A3" s="255" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="256" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="28" t="s">
@@ -26174,70 +26174,70 @@
       <c r="K3" s="28" t="s">
         <v>249</v>
       </c>
-      <c r="M3" s="258" t="s">
+      <c r="M3" s="260" t="s">
         <v>34</v>
       </c>
-      <c r="N3" s="204" t="s">
+      <c r="N3" s="202" t="s">
         <v>250</v>
       </c>
-      <c r="O3" s="205"/>
-      <c r="P3" s="205"/>
-      <c r="Q3" s="205"/>
-      <c r="R3" s="261" t="s">
+      <c r="O3" s="203"/>
+      <c r="P3" s="203"/>
+      <c r="Q3" s="203"/>
+      <c r="R3" s="253" t="s">
         <v>251</v>
       </c>
-      <c r="S3" s="204" t="s">
+      <c r="S3" s="202" t="s">
         <v>252</v>
       </c>
-      <c r="T3" s="205"/>
-      <c r="U3" s="205"/>
-      <c r="V3" s="205"/>
-      <c r="W3" s="261" t="s">
+      <c r="T3" s="203"/>
+      <c r="U3" s="203"/>
+      <c r="V3" s="203"/>
+      <c r="W3" s="253" t="s">
         <v>251</v>
       </c>
-      <c r="X3" s="207" t="s">
+      <c r="X3" s="215" t="s">
         <v>41</v>
       </c>
-      <c r="Y3" s="208"/>
-      <c r="Z3" s="208"/>
-      <c r="AA3" s="261" t="s">
+      <c r="Y3" s="216"/>
+      <c r="Z3" s="216"/>
+      <c r="AA3" s="253" t="s">
         <v>251</v>
       </c>
       <c r="AB3" s="71"/>
-      <c r="AC3" s="204" t="s">
+      <c r="AC3" s="202" t="s">
         <v>42</v>
       </c>
-      <c r="AD3" s="205"/>
-      <c r="AE3" s="205"/>
-      <c r="AF3" s="205"/>
-      <c r="AG3" s="204" t="s">
+      <c r="AD3" s="203"/>
+      <c r="AE3" s="203"/>
+      <c r="AF3" s="203"/>
+      <c r="AG3" s="202" t="s">
         <v>43</v>
       </c>
-      <c r="AH3" s="205"/>
-      <c r="AI3" s="205"/>
-      <c r="AJ3" s="205"/>
-      <c r="AK3" s="204" t="s">
+      <c r="AH3" s="203"/>
+      <c r="AI3" s="203"/>
+      <c r="AJ3" s="203"/>
+      <c r="AK3" s="202" t="s">
         <v>44</v>
       </c>
-      <c r="AL3" s="205"/>
-      <c r="AM3" s="205"/>
-      <c r="AN3" s="205"/>
-      <c r="AO3" s="204" t="s">
+      <c r="AL3" s="203"/>
+      <c r="AM3" s="203"/>
+      <c r="AN3" s="203"/>
+      <c r="AO3" s="202" t="s">
         <v>46</v>
       </c>
-      <c r="AP3" s="205"/>
-      <c r="AQ3" s="205"/>
-      <c r="AR3" s="205"/>
-      <c r="AS3" s="204" t="s">
+      <c r="AP3" s="203"/>
+      <c r="AQ3" s="203"/>
+      <c r="AR3" s="203"/>
+      <c r="AS3" s="202" t="s">
         <v>47</v>
       </c>
-      <c r="AT3" s="205"/>
-      <c r="AU3" s="205"/>
-      <c r="AV3" s="205"/>
+      <c r="AT3" s="203"/>
+      <c r="AU3" s="203"/>
+      <c r="AV3" s="203"/>
     </row>
     <row r="4" spans="1:48" ht="22.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="253"/>
-      <c r="B4" s="255"/>
+      <c r="A4" s="255"/>
+      <c r="B4" s="257"/>
       <c r="C4" s="24">
         <f t="shared" ref="C4:K4" si="0">SUM(C5:C19)</f>
         <v>15</v>
@@ -26274,7 +26274,7 @@
         <f t="shared" si="0"/>
         <v>134</v>
       </c>
-      <c r="M4" s="258"/>
+      <c r="M4" s="260"/>
       <c r="N4" s="8" t="s">
         <v>2</v>
       </c>
@@ -26287,7 +26287,7 @@
       <c r="Q4" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="R4" s="262"/>
+      <c r="R4" s="254"/>
       <c r="S4" s="8" t="s">
         <v>2</v>
       </c>
@@ -26300,7 +26300,7 @@
       <c r="V4" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="W4" s="262"/>
+      <c r="W4" s="254"/>
       <c r="X4" s="8" t="s">
         <v>2</v>
       </c>
@@ -26310,7 +26310,7 @@
       <c r="Z4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA4" s="262"/>
+      <c r="AA4" s="254"/>
       <c r="AB4" s="51" t="s">
         <v>59</v>
       </c>
@@ -28699,6 +28699,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A1:K2"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="N3:Q3"/>
+    <mergeCell ref="M1:Z2"/>
     <mergeCell ref="AS3:AV3"/>
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="W3:W4"/>
@@ -28709,12 +28715,6 @@
     <mergeCell ref="AK3:AN3"/>
     <mergeCell ref="AO3:AR3"/>
     <mergeCell ref="S3:V3"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A1:K2"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="N3:Q3"/>
-    <mergeCell ref="M1:Z2"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="P5:P20">
@@ -28854,44 +28854,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="263"/>
-      <c r="B1" s="263"/>
-      <c r="C1" s="263"/>
-      <c r="D1" s="263"/>
-      <c r="E1" s="263"/>
-      <c r="F1" s="263"/>
-      <c r="G1" s="263"/>
-      <c r="H1" s="263"/>
-      <c r="I1" s="263"/>
-      <c r="J1" s="263"/>
-      <c r="K1" s="263"/>
-      <c r="L1" s="263"/>
-      <c r="M1" s="263"/>
-      <c r="N1" s="263"/>
-      <c r="O1" s="263"/>
-      <c r="P1" s="263"/>
+      <c r="A1" s="265"/>
+      <c r="B1" s="265"/>
+      <c r="C1" s="265"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
+      <c r="F1" s="265"/>
+      <c r="G1" s="265"/>
+      <c r="H1" s="265"/>
+      <c r="I1" s="265"/>
+      <c r="J1" s="265"/>
+      <c r="K1" s="265"/>
+      <c r="L1" s="265"/>
+      <c r="M1" s="265"/>
+      <c r="N1" s="265"/>
+      <c r="O1" s="265"/>
+      <c r="P1" s="265"/>
     </row>
     <row r="2" spans="1:23" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="264"/>
-      <c r="B2" s="264"/>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
-      <c r="P2" s="264"/>
+      <c r="A2" s="266"/>
+      <c r="B2" s="266"/>
+      <c r="C2" s="266"/>
+      <c r="D2" s="266"/>
+      <c r="E2" s="266"/>
+      <c r="F2" s="266"/>
+      <c r="G2" s="266"/>
+      <c r="H2" s="266"/>
+      <c r="I2" s="266"/>
+      <c r="J2" s="266"/>
+      <c r="K2" s="266"/>
+      <c r="L2" s="266"/>
+      <c r="M2" s="266"/>
+      <c r="N2" s="266"/>
+      <c r="O2" s="266"/>
+      <c r="P2" s="266"/>
     </row>
     <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="265"/>
-      <c r="B3" s="265"/>
+      <c r="A3" s="267"/>
+      <c r="B3" s="267"/>
       <c r="C3" s="133"/>
       <c r="D3" s="133"/>
       <c r="E3" s="133"/>
@@ -28908,10 +28908,10 @@
       <c r="P3" s="133"/>
     </row>
     <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="267" t="s">
+      <c r="A4" s="269" t="s">
         <v>255</v>
       </c>
-      <c r="B4" s="267" t="s">
+      <c r="B4" s="269" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="141"/>
@@ -28919,70 +28919,70 @@
       <c r="E4" s="141"/>
       <c r="F4" s="141"/>
       <c r="G4" s="141"/>
-      <c r="H4" s="266"/>
-      <c r="I4" s="266"/>
-      <c r="J4" s="266"/>
-      <c r="K4" s="266"/>
-      <c r="L4" s="266"/>
-      <c r="M4" s="266"/>
-      <c r="N4" s="266"/>
-      <c r="O4" s="266"/>
-      <c r="P4" s="266"/>
+      <c r="H4" s="268"/>
+      <c r="I4" s="268"/>
+      <c r="J4" s="268"/>
+      <c r="K4" s="268"/>
+      <c r="L4" s="268"/>
+      <c r="M4" s="268"/>
+      <c r="N4" s="268"/>
+      <c r="O4" s="268"/>
+      <c r="P4" s="268"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.45">
-      <c r="A5" s="270"/>
-      <c r="B5" s="270"/>
-      <c r="C5" s="267" t="s">
+      <c r="A5" s="272"/>
+      <c r="B5" s="272"/>
+      <c r="C5" s="269" t="s">
         <v>256</v>
       </c>
-      <c r="D5" s="267" t="s">
+      <c r="D5" s="269" t="s">
         <v>257</v>
       </c>
-      <c r="E5" s="268"/>
-      <c r="F5" s="267" t="s">
+      <c r="E5" s="270"/>
+      <c r="F5" s="269" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="268"/>
-      <c r="H5" s="267" t="s">
+      <c r="G5" s="270"/>
+      <c r="H5" s="269" t="s">
         <v>259</v>
       </c>
-      <c r="I5" s="268"/>
-      <c r="J5" s="267" t="s">
+      <c r="I5" s="270"/>
+      <c r="J5" s="269" t="s">
         <v>260</v>
       </c>
-      <c r="K5" s="268"/>
-      <c r="L5" s="271" t="s">
+      <c r="K5" s="270"/>
+      <c r="L5" s="273" t="s">
         <v>261</v>
       </c>
-      <c r="M5" s="268"/>
-      <c r="N5" s="266" t="s">
+      <c r="M5" s="270"/>
+      <c r="N5" s="268" t="s">
         <v>262</v>
       </c>
-      <c r="O5" s="272"/>
-      <c r="P5" s="267" t="s">
+      <c r="O5" s="274"/>
+      <c r="P5" s="269" t="s">
         <v>266</v>
       </c>
-      <c r="R5" s="273" t="s">
+      <c r="R5" s="263" t="s">
         <v>34</v>
       </c>
-      <c r="S5" s="273" t="s">
+      <c r="S5" s="263" t="s">
         <v>290</v>
       </c>
-      <c r="T5" s="273" t="s">
+      <c r="T5" s="263" t="s">
         <v>291</v>
       </c>
-      <c r="U5" s="273" t="s">
+      <c r="U5" s="263" t="s">
         <v>293</v>
       </c>
-      <c r="V5" s="274" t="s">
+      <c r="V5" s="264" t="s">
         <v>292</v>
       </c>
       <c r="W5" s="172"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.45">
-      <c r="A6" s="269"/>
-      <c r="B6" s="269"/>
-      <c r="C6" s="270"/>
+      <c r="A6" s="271"/>
+      <c r="B6" s="271"/>
+      <c r="C6" s="272"/>
       <c r="D6" s="134" t="s">
         <v>2</v>
       </c>
@@ -29019,12 +29019,12 @@
       <c r="O6" s="134" t="s">
         <v>263</v>
       </c>
-      <c r="P6" s="269"/>
-      <c r="R6" s="273"/>
-      <c r="S6" s="273"/>
-      <c r="T6" s="273"/>
-      <c r="U6" s="273"/>
-      <c r="V6" s="273"/>
+      <c r="P6" s="271"/>
+      <c r="R6" s="263"/>
+      <c r="S6" s="263"/>
+      <c r="T6" s="263"/>
+      <c r="U6" s="263"/>
+      <c r="V6" s="263"/>
       <c r="W6" s="172"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.45">
@@ -29056,26 +29056,26 @@
         <v>72573808</v>
       </c>
       <c r="J7" s="191">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K7" s="191">
-        <v>509000</v>
+        <v>1270896</v>
       </c>
       <c r="L7" s="191">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="M7" s="191">
-        <v>59028396</v>
+        <v>59790292</v>
       </c>
       <c r="N7" s="192">
-        <v>83.18</v>
+        <v>84.1</v>
       </c>
       <c r="O7" s="192">
-        <v>81.34</v>
+        <v>82.39</v>
       </c>
       <c r="P7" s="135">
         <f>I7*0.97-M7</f>
-        <v>11368197.760000005</v>
+        <v>10606301.760000005</v>
       </c>
       <c r="R7" s="173" t="s">
         <v>117</v>
@@ -29089,11 +29089,11 @@
       </c>
       <c r="U7" s="189">
         <f>VLOOKUP(R7,$C$7:$P$27,14,0)</f>
-        <v>27733838.799999997</v>
+        <v>26057253.799999997</v>
       </c>
       <c r="V7" s="175">
         <f>VLOOKUP(R7,$C$7:$P$27,14,0)-T7</f>
-        <v>0</v>
+        <v>-1676585</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.45">
@@ -29125,26 +29125,26 @@
         <v>70243418</v>
       </c>
       <c r="J8" s="194">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K8" s="194">
-        <v>0</v>
+        <v>1586389</v>
       </c>
       <c r="L8" s="194">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="M8" s="194">
-        <v>55273476</v>
+        <v>56859865</v>
       </c>
       <c r="N8" s="195">
-        <v>76.430000000000007</v>
+        <v>78.849999999999994</v>
       </c>
       <c r="O8" s="195">
-        <v>78.69</v>
+        <v>80.95</v>
       </c>
       <c r="P8" s="135">
         <f t="shared" ref="P8:P27" si="0">I8*0.97-M8</f>
-        <v>12862639.459999993</v>
+        <v>11276250.459999993</v>
       </c>
       <c r="R8" s="173" t="s">
         <v>67</v>
@@ -29158,11 +29158,11 @@
       </c>
       <c r="U8" s="189">
         <f t="shared" ref="U8:U17" si="2">VLOOKUP(R8,$C$7:$P$27,14,0)</f>
-        <v>28033862.310000002</v>
+        <v>26149040.310000002</v>
       </c>
       <c r="V8" s="175">
         <f t="shared" ref="V8:V17" si="3">VLOOKUP(R8,$C$7:$P$27,14,0)-T8</f>
-        <v>0</v>
+        <v>-1884822</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.45">
@@ -29194,26 +29194,26 @@
         <v>145101823</v>
       </c>
       <c r="J9" s="191">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="K9" s="191">
-        <v>160000</v>
+        <v>2044822</v>
       </c>
       <c r="L9" s="191">
-        <v>660</v>
+        <v>672</v>
       </c>
       <c r="M9" s="191">
-        <v>112714906</v>
+        <v>114599728</v>
       </c>
       <c r="N9" s="192">
-        <v>75.34</v>
+        <v>76.709999999999994</v>
       </c>
       <c r="O9" s="192">
-        <v>77.680000000000007</v>
+        <v>78.98</v>
       </c>
       <c r="P9" s="135">
         <f t="shared" si="0"/>
-        <v>28033862.310000002</v>
+        <v>26149040.310000002</v>
       </c>
       <c r="R9" s="174" t="s">
         <v>87</v>
@@ -29227,11 +29227,11 @@
       </c>
       <c r="U9" s="189">
         <f t="shared" si="2"/>
-        <v>49090015.270000011</v>
+        <v>46511764.270000011</v>
       </c>
       <c r="V9" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-2578251</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.45">
@@ -29263,26 +29263,26 @@
         <v>51982396</v>
       </c>
       <c r="J10" s="194">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K10" s="194">
-        <v>100000</v>
+        <v>1258419</v>
       </c>
       <c r="L10" s="194">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="M10" s="194">
-        <v>39236420</v>
+        <v>40394839</v>
       </c>
       <c r="N10" s="195">
-        <v>75</v>
+        <v>77.27</v>
       </c>
       <c r="O10" s="195">
-        <v>75.48</v>
+        <v>77.709999999999994</v>
       </c>
       <c r="P10" s="135">
         <f t="shared" si="0"/>
-        <v>11186504.119999997</v>
+        <v>10028085.119999997</v>
       </c>
       <c r="R10" s="174" t="s">
         <v>110</v>
@@ -29296,28 +29296,28 @@
       </c>
       <c r="U10" s="189">
         <f t="shared" si="2"/>
-        <v>61083318.859999985</v>
+        <v>58912775.859999985</v>
       </c>
       <c r="V10" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-2170543</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A11" s="190" t="s">
-        <v>288</v>
+        <v>129</v>
       </c>
       <c r="B11" s="190" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C11" s="190" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D11" s="191">
-        <v>559</v>
+        <v>1048</v>
       </c>
       <c r="E11" s="191">
-        <v>93597302</v>
+        <v>180440547</v>
       </c>
       <c r="F11" s="191">
         <v>0</v>
@@ -29326,32 +29326,32 @@
         <v>0</v>
       </c>
       <c r="H11" s="191">
-        <v>559</v>
+        <v>1048</v>
       </c>
       <c r="I11" s="191">
-        <v>93597302</v>
+        <v>180440547</v>
       </c>
       <c r="J11" s="191">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="K11" s="191">
-        <v>558651</v>
+        <v>6929191</v>
       </c>
       <c r="L11" s="191">
-        <v>408</v>
+        <v>787</v>
       </c>
       <c r="M11" s="191">
-        <v>70116733</v>
+        <v>139450047</v>
       </c>
       <c r="N11" s="192">
-        <v>72.989999999999995</v>
+        <v>75.099999999999994</v>
       </c>
       <c r="O11" s="192">
-        <v>74.91</v>
+        <v>77.28</v>
       </c>
       <c r="P11" s="135">
         <f t="shared" si="0"/>
-        <v>20672649.939999998</v>
+        <v>35577283.590000004</v>
       </c>
       <c r="R11" s="173" t="s">
         <v>99</v>
@@ -29365,11 +29365,11 @@
       </c>
       <c r="U11" s="189">
         <f t="shared" si="2"/>
-        <v>41167886.75</v>
+        <v>40670886.75</v>
       </c>
       <c r="V11" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-497000</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.45">
@@ -29377,16 +29377,16 @@
         <v>288</v>
       </c>
       <c r="B12" s="193" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="C12" s="193" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="D12" s="194">
-        <v>716</v>
+        <v>559</v>
       </c>
       <c r="E12" s="194">
-        <v>116427734</v>
+        <v>93597302</v>
       </c>
       <c r="F12" s="194">
         <v>0</v>
@@ -29395,32 +29395,32 @@
         <v>0</v>
       </c>
       <c r="H12" s="194">
-        <v>716</v>
+        <v>559</v>
       </c>
       <c r="I12" s="194">
-        <v>116427734</v>
+        <v>93597302</v>
       </c>
       <c r="J12" s="194">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="K12" s="194">
-        <v>270000</v>
+        <v>2342270</v>
       </c>
       <c r="L12" s="194">
-        <v>516</v>
+        <v>420</v>
       </c>
       <c r="M12" s="194">
-        <v>87160486</v>
+        <v>71900352</v>
       </c>
       <c r="N12" s="195">
-        <v>72.069999999999993</v>
+        <v>75.13</v>
       </c>
       <c r="O12" s="195">
-        <v>74.86</v>
+        <v>76.819999999999993</v>
       </c>
       <c r="P12" s="135">
         <f t="shared" si="0"/>
-        <v>25774415.980000004</v>
+        <v>18889030.939999998</v>
       </c>
       <c r="R12" s="173" t="s">
         <v>75</v>
@@ -29434,28 +29434,28 @@
       </c>
       <c r="U12" s="189">
         <f t="shared" si="2"/>
-        <v>36430325.520000011</v>
+        <v>33601046.520000011</v>
       </c>
       <c r="V12" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-2829279</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A13" s="190" t="s">
-        <v>129</v>
+        <v>288</v>
       </c>
       <c r="B13" s="190" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="C13" s="190" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="D13" s="191">
-        <v>1181</v>
+        <v>716</v>
       </c>
       <c r="E13" s="191">
-        <v>189656153</v>
+        <v>116427734</v>
       </c>
       <c r="F13" s="191">
         <v>0</v>
@@ -29464,32 +29464,32 @@
         <v>0</v>
       </c>
       <c r="H13" s="191">
-        <v>1181</v>
+        <v>716</v>
       </c>
       <c r="I13" s="191">
-        <v>189656153</v>
+        <v>116427734</v>
       </c>
       <c r="J13" s="191">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="K13" s="191">
-        <v>757317</v>
+        <v>2087490</v>
       </c>
       <c r="L13" s="191">
-        <v>858</v>
+        <v>531</v>
       </c>
       <c r="M13" s="191">
-        <v>140517492</v>
+        <v>88977976</v>
       </c>
       <c r="N13" s="192">
-        <v>72.650000000000006</v>
+        <v>74.16</v>
       </c>
       <c r="O13" s="192">
-        <v>74.09</v>
+        <v>76.42</v>
       </c>
       <c r="P13" s="135">
         <f t="shared" si="0"/>
-        <v>43448976.409999996</v>
+        <v>23956925.980000004</v>
       </c>
       <c r="R13" s="173" t="s">
         <v>107</v>
@@ -29503,11 +29503,11 @@
       </c>
       <c r="U13" s="189">
         <f t="shared" si="2"/>
-        <v>41487079.590000004</v>
+        <v>35577283.590000004</v>
       </c>
       <c r="V13" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-5909796</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.45">
@@ -29515,16 +29515,16 @@
         <v>129</v>
       </c>
       <c r="B14" s="193" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C14" s="193" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D14" s="194">
-        <v>1048</v>
+        <v>1181</v>
       </c>
       <c r="E14" s="194">
-        <v>180440547</v>
+        <v>189656153</v>
       </c>
       <c r="F14" s="194">
         <v>0</v>
@@ -29533,32 +29533,32 @@
         <v>0</v>
       </c>
       <c r="H14" s="194">
-        <v>1048</v>
+        <v>1181</v>
       </c>
       <c r="I14" s="194">
-        <v>180440547</v>
+        <v>189656153</v>
       </c>
       <c r="J14" s="194">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="K14" s="194">
-        <v>1019395</v>
+        <v>4245520</v>
       </c>
       <c r="L14" s="194">
-        <v>752</v>
+        <v>875</v>
       </c>
       <c r="M14" s="194">
-        <v>133540251</v>
+        <v>144005695</v>
       </c>
       <c r="N14" s="195">
-        <v>71.760000000000005</v>
+        <v>74.09</v>
       </c>
       <c r="O14" s="195">
-        <v>74.010000000000005</v>
+        <v>75.930000000000007</v>
       </c>
       <c r="P14" s="135">
         <f t="shared" si="0"/>
-        <v>41487079.590000004</v>
+        <v>39960773.409999996</v>
       </c>
       <c r="R14" s="174" t="s">
         <v>72</v>
@@ -29572,11 +29572,11 @@
       </c>
       <c r="U14" s="189">
         <f t="shared" si="2"/>
-        <v>50987798.199999988</v>
+        <v>45616717.199999988</v>
       </c>
       <c r="V14" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-5371081</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.45">
@@ -29608,26 +29608,26 @@
         <v>152862316</v>
       </c>
       <c r="J15" s="191">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="K15" s="191">
-        <v>165123</v>
+        <v>2994402</v>
       </c>
       <c r="L15" s="191">
-        <v>649</v>
+        <v>670</v>
       </c>
       <c r="M15" s="191">
-        <v>111846121</v>
+        <v>114675400</v>
       </c>
       <c r="N15" s="192">
-        <v>68.97</v>
+        <v>71.2</v>
       </c>
       <c r="O15" s="192">
-        <v>73.17</v>
+        <v>75.02</v>
       </c>
       <c r="P15" s="135">
         <f t="shared" si="0"/>
-        <v>36430325.520000011</v>
+        <v>33601046.520000011</v>
       </c>
       <c r="R15" s="174" t="s">
         <v>113</v>
@@ -29641,11 +29641,11 @@
       </c>
       <c r="U15" s="189">
         <f t="shared" si="2"/>
-        <v>66475047.400000006</v>
+        <v>63603201.400000006</v>
       </c>
       <c r="V15" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-2871846</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.45">
@@ -29677,26 +29677,26 @@
         <v>66800107</v>
       </c>
       <c r="J16" s="194">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K16" s="194">
-        <v>451977</v>
+        <v>1193140</v>
       </c>
       <c r="L16" s="194">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="M16" s="194">
-        <v>48185464</v>
+        <v>48926627</v>
       </c>
       <c r="N16" s="195">
-        <v>68.67</v>
+        <v>70.12</v>
       </c>
       <c r="O16" s="195">
-        <v>72.13</v>
+        <v>73.239999999999995</v>
       </c>
       <c r="P16" s="135">
         <f t="shared" si="0"/>
-        <v>16610639.789999999</v>
+        <v>15869476.789999999</v>
       </c>
       <c r="R16" s="174" t="s">
         <v>119</v>
@@ -29710,11 +29710,11 @@
       </c>
       <c r="U16" s="189">
         <f t="shared" si="2"/>
-        <v>43448976.409999996</v>
+        <v>39960773.409999996</v>
       </c>
       <c r="V16" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-3488203</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.45">
@@ -29746,26 +29746,26 @@
         <v>53605661</v>
       </c>
       <c r="J17" s="191">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K17" s="191">
-        <v>355000</v>
+        <v>1499682</v>
       </c>
       <c r="L17" s="191">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="M17" s="191">
-        <v>37920198</v>
+        <v>39064880</v>
       </c>
       <c r="N17" s="192">
-        <v>66.290000000000006</v>
+        <v>68.260000000000005</v>
       </c>
       <c r="O17" s="192">
-        <v>70.739999999999995</v>
+        <v>72.87</v>
       </c>
       <c r="P17" s="135">
         <f t="shared" si="0"/>
-        <v>14077293.170000002</v>
+        <v>12932611.170000002</v>
       </c>
       <c r="R17" s="173" t="s">
         <v>84</v>
@@ -29779,11 +29779,11 @@
       </c>
       <c r="U17" s="189">
         <f t="shared" si="2"/>
-        <v>43417827.670000002</v>
+        <v>39390642.670000002</v>
       </c>
       <c r="V17" s="175">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-4027185</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.45">
@@ -29815,26 +29815,26 @@
         <v>101866340</v>
       </c>
       <c r="J18" s="194">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K18" s="194">
-        <v>0</v>
+        <v>1676585</v>
       </c>
       <c r="L18" s="194">
-        <v>428</v>
+        <v>439</v>
       </c>
       <c r="M18" s="194">
-        <v>71076511</v>
+        <v>72753096</v>
       </c>
       <c r="N18" s="195">
-        <v>66.67</v>
+        <v>68.38</v>
       </c>
       <c r="O18" s="195">
-        <v>69.77</v>
+        <v>71.42</v>
       </c>
       <c r="P18" s="135">
         <f t="shared" si="0"/>
-        <v>27733838.799999997</v>
+        <v>26057253.799999997</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.45">
@@ -29866,26 +29866,26 @@
         <v>50351985</v>
       </c>
       <c r="J19" s="191">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K19" s="191">
-        <v>0</v>
+        <v>830903</v>
       </c>
       <c r="L19" s="191">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="M19" s="191">
-        <v>34697236</v>
+        <v>35528139</v>
       </c>
       <c r="N19" s="192">
-        <v>65.72</v>
+        <v>67.3</v>
       </c>
       <c r="O19" s="192">
-        <v>68.91</v>
+        <v>70.56</v>
       </c>
       <c r="P19" s="135">
         <f t="shared" si="0"/>
-        <v>14144189.449999996</v>
+        <v>13313286.449999996</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.45">
@@ -29917,26 +29917,26 @@
         <v>162344260</v>
       </c>
       <c r="J20" s="194">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="K20" s="194">
-        <v>786437</v>
+        <v>6157518</v>
       </c>
       <c r="L20" s="194">
-        <v>631</v>
+        <v>655</v>
       </c>
       <c r="M20" s="194">
-        <v>106486134</v>
+        <v>111857215</v>
       </c>
       <c r="N20" s="195">
-        <v>65.19</v>
+        <v>67.67</v>
       </c>
       <c r="O20" s="195">
-        <v>65.59</v>
+        <v>68.900000000000006</v>
       </c>
       <c r="P20" s="135">
         <f t="shared" si="0"/>
-        <v>50987798.199999988</v>
+        <v>45616717.199999988</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.45">
@@ -29968,26 +29968,26 @@
         <v>194517020</v>
       </c>
       <c r="J21" s="191">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="K21" s="191">
-        <v>570329</v>
+        <v>3442175</v>
       </c>
       <c r="L21" s="191">
-        <v>735</v>
+        <v>753</v>
       </c>
       <c r="M21" s="191">
-        <v>122206462</v>
+        <v>125078308</v>
       </c>
       <c r="N21" s="192">
-        <v>61.35</v>
+        <v>62.85</v>
       </c>
       <c r="O21" s="192">
-        <v>62.83</v>
+        <v>64.3</v>
       </c>
       <c r="P21" s="135">
         <f t="shared" si="0"/>
-        <v>66475047.400000006</v>
+        <v>63603201.400000006</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.45">
@@ -30019,26 +30019,26 @@
         <v>141474291</v>
       </c>
       <c r="J22" s="194">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="K22" s="194">
-        <v>233432</v>
+        <v>2811683</v>
       </c>
       <c r="L22" s="194">
-        <v>523</v>
+        <v>536</v>
       </c>
       <c r="M22" s="194">
-        <v>88140047</v>
+        <v>90718298</v>
       </c>
       <c r="N22" s="195">
-        <v>61.31</v>
+        <v>62.84</v>
       </c>
       <c r="O22" s="195">
-        <v>62.3</v>
+        <v>64.12</v>
       </c>
       <c r="P22" s="135">
         <f t="shared" si="0"/>
-        <v>49090015.270000011</v>
+        <v>46511764.270000011</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.45">
@@ -30070,26 +30070,26 @@
         <v>105953075</v>
       </c>
       <c r="J23" s="191">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K23" s="191">
-        <v>0</v>
+        <v>497000</v>
       </c>
       <c r="L23" s="191">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="M23" s="191">
-        <v>61606596</v>
+        <v>62103596</v>
       </c>
       <c r="N23" s="192">
-        <v>56.91</v>
+        <v>57.64</v>
       </c>
       <c r="O23" s="192">
-        <v>58.15</v>
+        <v>58.61</v>
       </c>
       <c r="P23" s="135">
         <f t="shared" si="0"/>
-        <v>41167886.75</v>
+        <v>40670886.75</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.45">
@@ -30121,26 +30121,26 @@
         <v>149379338</v>
       </c>
       <c r="J24" s="194">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="K24" s="194">
-        <v>106494</v>
+        <v>2277037</v>
       </c>
       <c r="L24" s="194">
-        <v>506</v>
+        <v>518</v>
       </c>
       <c r="M24" s="194">
-        <v>83814639</v>
+        <v>85985182</v>
       </c>
       <c r="N24" s="195">
-        <v>56.73</v>
+        <v>58.07</v>
       </c>
       <c r="O24" s="195">
-        <v>56.11</v>
+        <v>57.56</v>
       </c>
       <c r="P24" s="135">
         <f t="shared" si="0"/>
-        <v>61083318.859999985</v>
+        <v>58912775.859999985</v>
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.45">
@@ -30172,26 +30172,26 @@
         <v>89879995</v>
       </c>
       <c r="J25" s="191">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="K25" s="191">
-        <v>185000</v>
+        <v>2253084</v>
       </c>
       <c r="L25" s="191">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="M25" s="191">
-        <v>49044586</v>
+        <v>51112670</v>
       </c>
       <c r="N25" s="192">
-        <v>52.56</v>
+        <v>54.76</v>
       </c>
       <c r="O25" s="192">
-        <v>54.57</v>
+        <v>56.87</v>
       </c>
       <c r="P25" s="135">
         <f t="shared" si="0"/>
-        <v>38139009.149999991</v>
+        <v>36070925.149999991</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.45">
@@ -30223,26 +30223,26 @@
         <v>95369711</v>
       </c>
       <c r="J26" s="194">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="K26" s="194">
-        <v>100000</v>
+        <v>4127185</v>
       </c>
       <c r="L26" s="194">
-        <v>292</v>
+        <v>317</v>
       </c>
       <c r="M26" s="194">
-        <v>49090792</v>
+        <v>53117977</v>
       </c>
       <c r="N26" s="195">
-        <v>49.66</v>
+        <v>53.91</v>
       </c>
       <c r="O26" s="195">
-        <v>51.47</v>
+        <v>55.7</v>
       </c>
       <c r="P26" s="135">
         <f t="shared" si="0"/>
-        <v>43417827.670000002</v>
+        <v>39390642.670000002</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.45">
@@ -30274,35 +30274,30 @@
         <v>105983346</v>
       </c>
       <c r="J27" s="191">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K27" s="191">
-        <v>0</v>
+        <v>932012</v>
       </c>
       <c r="L27" s="191">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="M27" s="191">
-        <v>32622142</v>
+        <v>33554154</v>
       </c>
       <c r="N27" s="192">
-        <v>30.89</v>
+        <v>31.77</v>
       </c>
       <c r="O27" s="192">
-        <v>30.78</v>
+        <v>31.66</v>
       </c>
       <c r="P27" s="135">
         <f t="shared" si="0"/>
-        <v>70181703.61999999</v>
+        <v>69249691.61999999</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="V5:V6"/>
-    <mergeCell ref="R5:R6"/>
-    <mergeCell ref="S5:S6"/>
-    <mergeCell ref="T5:T6"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A3:B3"/>
@@ -30317,6 +30312,11 @@
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="L5:M5"/>
     <mergeCell ref="N5:O5"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="V5:V6"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="S5:S6"/>
+    <mergeCell ref="T5:T6"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="P7:P27">

</xml_diff>